<commit_message>
1000% dP error wheeee
</commit_message>
<xml_diff>
--- a/Drill_Bits.xlsx
+++ b/Drill_Bits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanchit Arora\Documents\GitHub\RocketSizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FADB167F-A9CC-45F5-A313-3EB3E264BB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192FB773-EFF2-45FD-9C9A-D92A69D2E0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{30BA82C0-201C-4D79-BA4E-B626623364AF}"/>
   </bookViews>
@@ -561,7 +561,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:C36" si="0">B3*25.4</f>
+        <f t="shared" ref="C3:C34" si="0">B3*25.4</f>
         <v>0.33019999999999999</v>
       </c>
     </row>
@@ -932,7 +932,7 @@
         <v>7.85E-2</v>
       </c>
       <c r="C35">
-        <f t="shared" si="0"/>
+        <f>B35*25.4</f>
         <v>1.9939</v>
       </c>
     </row>

</xml_diff>

<commit_message>
when is NOs liquid ;-;
</commit_message>
<xml_diff>
--- a/Drill_Bits.xlsx
+++ b/Drill_Bits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanchit Arora\Documents\GitHub\RocketSizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192FB773-EFF2-45FD-9C9A-D92A69D2E0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF849FBD-6090-487E-968A-B044AE550BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{30BA82C0-201C-4D79-BA4E-B626623364AF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{30BA82C0-201C-4D79-BA4E-B626623364AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>Drill Bit</t>
   </si>
@@ -150,6 +150,87 @@
   </si>
   <si>
     <t>2mm HSS</t>
+  </si>
+  <si>
+    <t>#46 HSS</t>
+  </si>
+  <si>
+    <t>#45 HSS</t>
+  </si>
+  <si>
+    <t>2.1mm HSS</t>
+  </si>
+  <si>
+    <t>#44 HSS</t>
+  </si>
+  <si>
+    <t>2.2mm HSS</t>
+  </si>
+  <si>
+    <t>#43 HSS</t>
+  </si>
+  <si>
+    <t>2.3mm HSS</t>
+  </si>
+  <si>
+    <t>#42 HSS</t>
+  </si>
+  <si>
+    <t>3/32" HSS</t>
+  </si>
+  <si>
+    <t>2.4mm HSS</t>
+  </si>
+  <si>
+    <t>#41 HSS</t>
+  </si>
+  <si>
+    <t>#40 HSS</t>
+  </si>
+  <si>
+    <t>2.5mm HSS</t>
+  </si>
+  <si>
+    <t>#39 HSS</t>
+  </si>
+  <si>
+    <t>#38 HSS</t>
+  </si>
+  <si>
+    <t>2.6mm HSS</t>
+  </si>
+  <si>
+    <t>#37 HSS</t>
+  </si>
+  <si>
+    <t>2.7mm HSS</t>
+  </si>
+  <si>
+    <t>#36 HSS</t>
+  </si>
+  <si>
+    <t>7/64" HSS</t>
+  </si>
+  <si>
+    <t>#35 HSS</t>
+  </si>
+  <si>
+    <t>2.8mm HSS</t>
+  </si>
+  <si>
+    <t>#34 HSS</t>
+  </si>
+  <si>
+    <t>#33 HSS</t>
+  </si>
+  <si>
+    <t>2.9mm HSS</t>
+  </si>
+  <si>
+    <t>#32 HSS</t>
+  </si>
+  <si>
+    <t>3mm HSS</t>
   </si>
 </sst>
 </file>
@@ -521,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F1C826-8A1E-49E5-A18A-9BF0C23C3712}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" customWidth="1"/>
@@ -947,7 +1028,332 @@
         <v>2</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37">
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="C37">
+        <f>B37*25.4</f>
+        <v>2.0573999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="C38">
+        <f>B38*25.4</f>
+        <v>2.0827999999999998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39">
+        <f>C39/25.4</f>
+        <v>8.2677165354330714E-2</v>
+      </c>
+      <c r="C39">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="C40">
+        <f>B40*25.4</f>
+        <v>2.1843999999999997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41">
+        <f>C41/25.4</f>
+        <v>8.6614173228346469E-2</v>
+      </c>
+      <c r="C41">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="C42">
+        <f>B42*25.4</f>
+        <v>2.2605999999999997</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43">
+        <f>C43/25.4</f>
+        <v>9.0551181102362197E-2</v>
+      </c>
+      <c r="C43">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44">
+        <v>9.35E-2</v>
+      </c>
+      <c r="C44">
+        <f>B44*25.4</f>
+        <v>2.3748999999999998</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45">
+        <v>9.375E-2</v>
+      </c>
+      <c r="C45">
+        <f>B45*25.4</f>
+        <v>2.3812499999999996</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46">
+        <f>C46/25.4</f>
+        <v>9.4488188976377951E-2</v>
+      </c>
+      <c r="C46">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="C47">
+        <f>B47*25.4</f>
+        <v>2.4384000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>49</v>
+      </c>
+      <c r="B48">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="C48">
+        <f>B48*25.4</f>
+        <v>2.4891999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49">
+        <f>C49/25.4</f>
+        <v>9.8425196850393706E-2</v>
+      </c>
+      <c r="C49">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>51</v>
+      </c>
+      <c r="B50">
+        <v>9.9500000000000005E-2</v>
+      </c>
+      <c r="C50">
+        <f>B49*25.4</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51">
+        <v>0.10150000000000001</v>
+      </c>
+      <c r="C51">
+        <f>B50*25.4</f>
+        <v>2.5272999999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>53</v>
+      </c>
+      <c r="B52">
+        <f>C52/25.4</f>
+        <v>0.10236220472440946</v>
+      </c>
+      <c r="C52">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>54</v>
+      </c>
+      <c r="B53">
+        <v>0.104</v>
+      </c>
+      <c r="C53">
+        <f>B52*25.4</f>
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>55</v>
+      </c>
+      <c r="B54">
+        <f>C54/25.4</f>
+        <v>0.10629921259842522</v>
+      </c>
+      <c r="C54">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>56</v>
+      </c>
+      <c r="B55">
+        <v>0.1065</v>
+      </c>
+      <c r="C55">
+        <f>B55*25.4</f>
+        <v>2.7050999999999998</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>57</v>
+      </c>
+      <c r="B56">
+        <v>0.109375</v>
+      </c>
+      <c r="C56">
+        <f t="shared" ref="C56:C57" si="1">B56*25.4</f>
+        <v>2.7781249999999997</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>58</v>
+      </c>
+      <c r="B57">
+        <v>0.11</v>
+      </c>
+      <c r="C57">
+        <f t="shared" si="1"/>
+        <v>2.794</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58">
+        <f>C58/25.4</f>
+        <v>0.11023622047244094</v>
+      </c>
+      <c r="C58">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59">
+        <v>0.111</v>
+      </c>
+      <c r="C59">
+        <f>B59*25.4</f>
+        <v>2.8193999999999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60">
+        <v>0.113</v>
+      </c>
+      <c r="C60">
+        <f>B60*25.4</f>
+        <v>2.8702000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61">
+        <f>C61/25.4</f>
+        <v>0.1141732283464567</v>
+      </c>
+      <c r="C61">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>63</v>
+      </c>
+      <c r="B62">
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="C62">
+        <f>B62*25.4</f>
+        <v>2.9464000000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>64</v>
+      </c>
+      <c r="B63">
+        <f>C63/25.4</f>
+        <v>0.11811023622047245</v>
+      </c>
+      <c r="C63">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>